<commit_message>
Fix unified-control.sh sed errors and test end-to-end grading with network capture
Co-authored-by: dongnuc <136960214+dongnuc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchstudent/Results/cuongnvhe181200/OverallSummary.xlsx
+++ b/batchstudent/Results/cuongnvhe181200/OverallSummary.xlsx
@@ -37,25 +37,25 @@
     <x:t>FAIL</x:t>
   </x:si>
   <x:si>
-    <x:t>Network monitoring failed: No packets captured. Run with sudo and ensure libpcap/NPcap is installed.; Network flows: 2 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
+    <x:t>Network flows: 2 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC2</x:t>
   </x:si>
   <x:si>
-    <x:t>Network monitoring failed: No packets captured. Run with sudo and ensure libpcap/NPcap is installed.; Network flows: 3 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
+    <x:t>Network flows: 3 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC3</x:t>
   </x:si>
   <x:si>
-    <x:t>Network monitoring failed: No packets captured. Run with sudo and ensure libpcap/NPcap is installed.; Network flows: 7 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
+    <x:t>Network flows: 7 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC4</x:t>
   </x:si>
   <x:si>
-    <x:t>Network monitoring failed: No packets captured. Run with sudo and ensure libpcap/NPcap is installed.; Network flows: 11 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
+    <x:t>Network flows: 11 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC5</x:t>
@@ -64,7 +64,7 @@
     <x:t>TC6</x:t>
   </x:si>
   <x:si>
-    <x:t>Network monitoring failed: No packets captured. Run with sudo and ensure libpcap/NPcap is installed.; Network flows: 22 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
+    <x:t>Network flows: 22 FAIL (ALL-OR-NOTHING: test FAILED), 0 PARTIAL, 0 PASS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -437,7 +437,7 @@
     <x:col min="2" max="2" width="7.282054" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="159.853482" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="66.567768" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:5" s="1" customFormat="1">

</xml_diff>